<commit_message>
Self-audit fixes: code-fallback, no phantom img, stable upload name
#1 (regression) 수식 셀이 미계산이면 import 시 문항코드 빈값 →
  bulk-parse/route.ts·question_io.py 에 출처 기반 문항코드 재계산 폴백 추가.
  샘플 행은 문항코드 정적값으로 환원(import 안전). E2E 검증 완료.
#2 엑셀 이미지명 자동수식 제거 (유령 src 방지) — 이미지명은 업로드가 부여.
#3 upload/route.ts 재업로드 시 _2 suffix → 덮어쓰기로 변경(규칙 파일명 고정).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/샘플_2022_1회_v1.xlsx
+++ b/data/templates/샘플_2022_1회_v1.xlsx
@@ -200,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -275,9 +275,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -947,9 +944,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G3" s="26">
-        <f>IF(COUNTA($F3,$B3,$C3,$D3)=4,"elec_"&amp;$F3&amp;"_"&amp;$B3&amp;"_"&amp;TEXT($C3,"00")&amp;"_"&amp;TEXT($D3,"00"),"")</f>
-        <v/>
+      <c r="G3" s="25" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_01</t>
+        </is>
       </c>
       <c r="H3" s="24" t="inlineStr"/>
       <c r="I3" s="24" t="inlineStr">
@@ -1073,9 +1071,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G4" s="26">
-        <f>IF(COUNTA($F4,$B4,$C4,$D4)=4,"elec_"&amp;$F4&amp;"_"&amp;$B4&amp;"_"&amp;TEXT($C4,"00")&amp;"_"&amp;TEXT($D4,"00"),"")</f>
-        <v/>
+      <c r="G4" s="25" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_02</t>
+        </is>
       </c>
       <c r="H4" s="24" t="inlineStr"/>
       <c r="I4" s="24" t="inlineStr">
@@ -1189,9 +1188,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G5" s="26">
-        <f>IF(COUNTA($F5,$B5,$C5,$D5)=4,"elec_"&amp;$F5&amp;"_"&amp;$B5&amp;"_"&amp;TEXT($C5,"00")&amp;"_"&amp;TEXT($D5,"00"),"")</f>
-        <v/>
+      <c r="G5" s="25" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_05</t>
+        </is>
       </c>
       <c r="H5" s="24" t="inlineStr"/>
       <c r="I5" s="24" t="inlineStr">
@@ -1305,9 +1305,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G6" s="26">
-        <f>IF(COUNTA($F6,$B6,$C6,$D6)=4,"elec_"&amp;$F6&amp;"_"&amp;$B6&amp;"_"&amp;TEXT($C6,"00")&amp;"_"&amp;TEXT($D6,"00"),"")</f>
-        <v/>
+      <c r="G6" s="25" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_07</t>
+        </is>
       </c>
       <c r="H6" s="24" t="inlineStr"/>
       <c r="I6" s="24" t="inlineStr">
@@ -1426,9 +1427,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G7" s="26">
-        <f>IF(COUNTA($F7,$B7,$C7,$D7)=4,"elec_"&amp;$F7&amp;"_"&amp;$B7&amp;"_"&amp;TEXT($C7,"00")&amp;"_"&amp;TEXT($D7,"00"),"")</f>
-        <v/>
+      <c r="G7" s="25" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_11</t>
+        </is>
       </c>
       <c r="H7" s="24" t="inlineStr"/>
       <c r="I7" s="24" t="inlineStr">
@@ -1548,9 +1550,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G8" s="26">
-        <f>IF(COUNTA($F8,$B8,$C8,$D8)=4,"elec_"&amp;$F8&amp;"_"&amp;$B8&amp;"_"&amp;TEXT($C8,"00")&amp;"_"&amp;TEXT($D8,"00"),"")</f>
-        <v/>
+      <c r="G8" s="25" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_13</t>
+        </is>
       </c>
       <c r="H8" s="24" t="inlineStr"/>
       <c r="I8" s="24" t="inlineStr">
@@ -1669,9 +1672,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G9" s="26">
-        <f>IF(COUNTA($F9,$B9,$C9,$D9)=4,"elec_"&amp;$F9&amp;"_"&amp;$B9&amp;"_"&amp;TEXT($C9,"00")&amp;"_"&amp;TEXT($D9,"00"),"")</f>
-        <v/>
+      <c r="G9" s="25" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_23</t>
+        </is>
       </c>
       <c r="H9" s="24" t="inlineStr"/>
       <c r="I9" s="25" t="inlineStr">
@@ -1796,9 +1800,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G10" s="26">
-        <f>IF(COUNTA($F10,$B10,$C10,$D10)=4,"elec_"&amp;$F10&amp;"_"&amp;$B10&amp;"_"&amp;TEXT($C10,"00")&amp;"_"&amp;TEXT($D10,"00"),"")</f>
-        <v/>
+      <c r="G10" s="25" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_32</t>
+        </is>
       </c>
       <c r="H10" s="24" t="inlineStr"/>
       <c r="I10" s="25" t="inlineStr">
@@ -1917,9 +1922,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G11" s="26">
-        <f>IF(COUNTA($F11,$B11,$C11,$D11)=4,"elec_"&amp;$F11&amp;"_"&amp;$B11&amp;"_"&amp;TEXT($C11,"00")&amp;"_"&amp;TEXT($D11,"00"),"")</f>
-        <v/>
+      <c r="G11" s="25" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_39</t>
+        </is>
       </c>
       <c r="H11" s="24" t="inlineStr"/>
       <c r="I11" s="24" t="inlineStr">
@@ -2039,9 +2045,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G12" s="26">
-        <f>IF(COUNTA($F12,$B12,$C12,$D12)=4,"elec_"&amp;$F12&amp;"_"&amp;$B12&amp;"_"&amp;TEXT($C12,"00")&amp;"_"&amp;TEXT($D12,"00"),"")</f>
-        <v/>
+      <c r="G12" s="25" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_60</t>
+        </is>
       </c>
       <c r="H12" s="24" t="inlineStr"/>
       <c r="I12" s="24" t="inlineStr">
@@ -2151,7 +2158,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="26">
         <f>IF(COUNTA($F13,$B13,$C13,$D13)=4,"elec_"&amp;$F13&amp;"_"&amp;$B13&amp;"_"&amp;TEXT($C13,"00")&amp;"_"&amp;TEXT($D13,"00"),"")</f>
         <v/>
       </c>
@@ -2167,35 +2174,20 @@
       <c r="Q13" s="24" t="inlineStr"/>
       <c r="R13" s="25" t="inlineStr">
         <is>
-          <t>← 출처만 채운 데모행: 코드·이미지명 자동 생성됨</t>
+          <t>← 출처만 채운 데모행: 문항코드 자동 생성됨</t>
         </is>
       </c>
       <c r="S13" s="25" t="inlineStr"/>
       <c r="T13" s="24" t="inlineStr"/>
-      <c r="U13" s="27">
-        <f>IF($G13="","",$G13&amp;"_stem1.png")</f>
-        <v/>
-      </c>
+      <c r="U13" s="24" t="inlineStr"/>
       <c r="V13" s="24" t="inlineStr"/>
-      <c r="W13" s="27">
-        <f>IF($G13="","",$G13&amp;"_opt1.png")</f>
-        <v/>
-      </c>
+      <c r="W13" s="24" t="inlineStr"/>
       <c r="X13" s="24" t="inlineStr"/>
-      <c r="Y13" s="27">
-        <f>IF($G13="","",$G13&amp;"_opt2.png")</f>
-        <v/>
-      </c>
+      <c r="Y13" s="24" t="inlineStr"/>
       <c r="Z13" s="24" t="inlineStr"/>
-      <c r="AA13" s="27">
-        <f>IF($G13="","",$G13&amp;"_opt3.png")</f>
-        <v/>
-      </c>
+      <c r="AA13" s="24" t="inlineStr"/>
       <c r="AB13" s="24" t="inlineStr"/>
-      <c r="AC13" s="27">
-        <f>IF($G13="","",$G13&amp;"_opt4.png")</f>
-        <v/>
-      </c>
+      <c r="AC13" s="24" t="inlineStr"/>
       <c r="AD13" s="24" t="inlineStr"/>
       <c r="AE13" s="24" t="inlineStr"/>
       <c r="AF13" s="24" t="inlineStr"/>
@@ -2208,7 +2200,7 @@
       <c r="D14" s="24" t="inlineStr"/>
       <c r="E14" s="24" t="inlineStr"/>
       <c r="F14" s="24" t="inlineStr"/>
-      <c r="G14" s="27">
+      <c r="G14" s="26">
         <f>IF(COUNTA($F14,$B14,$C14,$D14)=4,"elec_"&amp;$F14&amp;"_"&amp;$B14&amp;"_"&amp;TEXT($C14,"00")&amp;"_"&amp;TEXT($D14,"00"),"")</f>
         <v/>
       </c>
@@ -2225,30 +2217,15 @@
       <c r="R14" s="25" t="inlineStr"/>
       <c r="S14" s="25" t="inlineStr"/>
       <c r="T14" s="24" t="inlineStr"/>
-      <c r="U14" s="27">
-        <f>IF($G14="","",$G14&amp;"_stem1.png")</f>
-        <v/>
-      </c>
+      <c r="U14" s="24" t="inlineStr"/>
       <c r="V14" s="24" t="inlineStr"/>
-      <c r="W14" s="27">
-        <f>IF($G14="","",$G14&amp;"_opt1.png")</f>
-        <v/>
-      </c>
+      <c r="W14" s="24" t="inlineStr"/>
       <c r="X14" s="24" t="inlineStr"/>
-      <c r="Y14" s="27">
-        <f>IF($G14="","",$G14&amp;"_opt2.png")</f>
-        <v/>
-      </c>
+      <c r="Y14" s="24" t="inlineStr"/>
       <c r="Z14" s="24" t="inlineStr"/>
-      <c r="AA14" s="27">
-        <f>IF($G14="","",$G14&amp;"_opt3.png")</f>
-        <v/>
-      </c>
+      <c r="AA14" s="24" t="inlineStr"/>
       <c r="AB14" s="24" t="inlineStr"/>
-      <c r="AC14" s="27">
-        <f>IF($G14="","",$G14&amp;"_opt4.png")</f>
-        <v/>
-      </c>
+      <c r="AC14" s="24" t="inlineStr"/>
       <c r="AD14" s="24" t="inlineStr"/>
       <c r="AE14" s="24" t="inlineStr"/>
       <c r="AF14" s="24" t="inlineStr"/>
@@ -2261,7 +2238,7 @@
       <c r="D15" s="24" t="inlineStr"/>
       <c r="E15" s="24" t="inlineStr"/>
       <c r="F15" s="24" t="inlineStr"/>
-      <c r="G15" s="27">
+      <c r="G15" s="26">
         <f>IF(COUNTA($F15,$B15,$C15,$D15)=4,"elec_"&amp;$F15&amp;"_"&amp;$B15&amp;"_"&amp;TEXT($C15,"00")&amp;"_"&amp;TEXT($D15,"00"),"")</f>
         <v/>
       </c>
@@ -2278,30 +2255,15 @@
       <c r="R15" s="25" t="inlineStr"/>
       <c r="S15" s="25" t="inlineStr"/>
       <c r="T15" s="24" t="inlineStr"/>
-      <c r="U15" s="27">
-        <f>IF($G15="","",$G15&amp;"_stem1.png")</f>
-        <v/>
-      </c>
+      <c r="U15" s="24" t="inlineStr"/>
       <c r="V15" s="24" t="inlineStr"/>
-      <c r="W15" s="27">
-        <f>IF($G15="","",$G15&amp;"_opt1.png")</f>
-        <v/>
-      </c>
+      <c r="W15" s="24" t="inlineStr"/>
       <c r="X15" s="24" t="inlineStr"/>
-      <c r="Y15" s="27">
-        <f>IF($G15="","",$G15&amp;"_opt2.png")</f>
-        <v/>
-      </c>
+      <c r="Y15" s="24" t="inlineStr"/>
       <c r="Z15" s="24" t="inlineStr"/>
-      <c r="AA15" s="27">
-        <f>IF($G15="","",$G15&amp;"_opt3.png")</f>
-        <v/>
-      </c>
+      <c r="AA15" s="24" t="inlineStr"/>
       <c r="AB15" s="24" t="inlineStr"/>
-      <c r="AC15" s="27">
-        <f>IF($G15="","",$G15&amp;"_opt4.png")</f>
-        <v/>
-      </c>
+      <c r="AC15" s="24" t="inlineStr"/>
       <c r="AD15" s="24" t="inlineStr"/>
       <c r="AE15" s="24" t="inlineStr"/>
       <c r="AF15" s="24" t="inlineStr"/>
@@ -2314,7 +2276,7 @@
       <c r="D16" s="24" t="inlineStr"/>
       <c r="E16" s="24" t="inlineStr"/>
       <c r="F16" s="24" t="inlineStr"/>
-      <c r="G16" s="27">
+      <c r="G16" s="26">
         <f>IF(COUNTA($F16,$B16,$C16,$D16)=4,"elec_"&amp;$F16&amp;"_"&amp;$B16&amp;"_"&amp;TEXT($C16,"00")&amp;"_"&amp;TEXT($D16,"00"),"")</f>
         <v/>
       </c>
@@ -2331,30 +2293,15 @@
       <c r="R16" s="25" t="inlineStr"/>
       <c r="S16" s="25" t="inlineStr"/>
       <c r="T16" s="24" t="inlineStr"/>
-      <c r="U16" s="27">
-        <f>IF($G16="","",$G16&amp;"_stem1.png")</f>
-        <v/>
-      </c>
+      <c r="U16" s="24" t="inlineStr"/>
       <c r="V16" s="24" t="inlineStr"/>
-      <c r="W16" s="27">
-        <f>IF($G16="","",$G16&amp;"_opt1.png")</f>
-        <v/>
-      </c>
+      <c r="W16" s="24" t="inlineStr"/>
       <c r="X16" s="24" t="inlineStr"/>
-      <c r="Y16" s="27">
-        <f>IF($G16="","",$G16&amp;"_opt2.png")</f>
-        <v/>
-      </c>
+      <c r="Y16" s="24" t="inlineStr"/>
       <c r="Z16" s="24" t="inlineStr"/>
-      <c r="AA16" s="27">
-        <f>IF($G16="","",$G16&amp;"_opt3.png")</f>
-        <v/>
-      </c>
+      <c r="AA16" s="24" t="inlineStr"/>
       <c r="AB16" s="24" t="inlineStr"/>
-      <c r="AC16" s="27">
-        <f>IF($G16="","",$G16&amp;"_opt4.png")</f>
-        <v/>
-      </c>
+      <c r="AC16" s="24" t="inlineStr"/>
       <c r="AD16" s="24" t="inlineStr"/>
       <c r="AE16" s="24" t="inlineStr"/>
       <c r="AF16" s="24" t="inlineStr"/>
@@ -2367,7 +2314,7 @@
       <c r="D17" s="24" t="inlineStr"/>
       <c r="E17" s="24" t="inlineStr"/>
       <c r="F17" s="24" t="inlineStr"/>
-      <c r="G17" s="27">
+      <c r="G17" s="26">
         <f>IF(COUNTA($F17,$B17,$C17,$D17)=4,"elec_"&amp;$F17&amp;"_"&amp;$B17&amp;"_"&amp;TEXT($C17,"00")&amp;"_"&amp;TEXT($D17,"00"),"")</f>
         <v/>
       </c>
@@ -2384,30 +2331,15 @@
       <c r="R17" s="25" t="inlineStr"/>
       <c r="S17" s="25" t="inlineStr"/>
       <c r="T17" s="24" t="inlineStr"/>
-      <c r="U17" s="27">
-        <f>IF($G17="","",$G17&amp;"_stem1.png")</f>
-        <v/>
-      </c>
+      <c r="U17" s="24" t="inlineStr"/>
       <c r="V17" s="24" t="inlineStr"/>
-      <c r="W17" s="27">
-        <f>IF($G17="","",$G17&amp;"_opt1.png")</f>
-        <v/>
-      </c>
+      <c r="W17" s="24" t="inlineStr"/>
       <c r="X17" s="24" t="inlineStr"/>
-      <c r="Y17" s="27">
-        <f>IF($G17="","",$G17&amp;"_opt2.png")</f>
-        <v/>
-      </c>
+      <c r="Y17" s="24" t="inlineStr"/>
       <c r="Z17" s="24" t="inlineStr"/>
-      <c r="AA17" s="27">
-        <f>IF($G17="","",$G17&amp;"_opt3.png")</f>
-        <v/>
-      </c>
+      <c r="AA17" s="24" t="inlineStr"/>
       <c r="AB17" s="24" t="inlineStr"/>
-      <c r="AC17" s="27">
-        <f>IF($G17="","",$G17&amp;"_opt4.png")</f>
-        <v/>
-      </c>
+      <c r="AC17" s="24" t="inlineStr"/>
       <c r="AD17" s="24" t="inlineStr"/>
       <c r="AE17" s="24" t="inlineStr"/>
       <c r="AF17" s="24" t="inlineStr"/>
@@ -2439,510 +2371,511 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>CBT 문항 콘텐츠 작성 규칙 (v1)</t>
         </is>
       </c>
-      <c r="B1" s="29" t="inlineStr"/>
+      <c r="B1" s="28" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="inlineStr"/>
-      <c r="B2" s="31" t="inlineStr"/>
+      <c r="A2" s="29" t="inlineStr"/>
+      <c r="B2" s="30" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>[문항코드 규칙]</t>
         </is>
       </c>
-      <c r="B3" s="29" t="inlineStr"/>
+      <c r="B3" s="28" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>형식</t>
         </is>
       </c>
-      <c r="B4" s="31" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>elec_&lt;교재구분&gt;_&lt;연도&gt;_&lt;회차2자리&gt;_&lt;번호2자리&gt;</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
-      <c r="B5" s="31" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>elec_A_2022_01_01  (교재 A · 2022년 · 1회 · 1번)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-      <c r="B6" s="31" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>정렬·식별 키.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="inlineStr"/>
-      <c r="B7" s="31" t="inlineStr"/>
+      <c r="A7" s="29" t="inlineStr"/>
+      <c r="B7" s="30" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
-        <is>
-          <t>[자동 생성 — 엑셀 수식]</t>
-        </is>
-      </c>
-      <c r="B8" s="29" t="inlineStr"/>
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>[자동 생성 — 문항코드]</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
-        <is>
-          <t>동작</t>
-        </is>
-      </c>
-      <c r="B9" s="31" t="inlineStr">
-        <is>
-          <t>출처(교재구분·연도·회차·번호)만 채우면 「문항코드」와 「발문/보기 그림」 셀이 수식으로 자동 형성</t>
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>샘플(3~12행)</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>문항코드 = 정적값(고정). 그대로 import 안전.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>자동 셀</t>
-        </is>
-      </c>
-      <c r="B10" s="31" t="inlineStr">
-        <is>
-          <t>연노랑 배경 = 수식 셀(직접 입력 금지). 13행~ = 빈 작성행(데모 포함)</t>
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>작성행(13행~)</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>문항코드 = 수식(연노랑). 출처만 채우면 즉시 표시 — 작성 편의용.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>문항코드</t>
-        </is>
-      </c>
-      <c r="B11" s="31">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>수식</t>
+        </is>
+      </c>
+      <c r="B11" s="30">
         <f>IF(COUNTA(...)=4,"elec_"&amp;교재구분&amp;"_"&amp;연도&amp;"_"&amp;TEXT(회차,"00")&amp;"_"&amp;TEXT(번호,"00"),"")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>안전장치</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>엑셀 수식은 저장 전 미계산일 수 있으나, 서버(일괄등록)가 출처로 문항코드를 재계산하므로 비어도 안전.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>이미지명</t>
         </is>
       </c>
-      <c r="B12" s="31">
-        <f>IF(문항코드="","",문항코드&amp;"_stem1.png")  (보기는 _opt1~4.png)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="30" t="inlineStr">
-        <is>
-          <t>주의</t>
-        </is>
-      </c>
-      <c r="B13" s="31" t="inlineStr">
-        <is>
-          <t>해당 슬롯에 그림이 없으면 그 이미지 셀 내용을 지운다(수식 덮어쓰기). 해설/학습포인트 안 그림은 본문에 &lt;img src="문항코드_exp1.png"&gt; 식으로.</t>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>엑셀에서 자동 생성하지 않음. 그림 업로드 시 서버가 {문항코드}_{슬롯}{순번}.png 로 부여(고정). 본문/그림셀엔 그 이름을 그대로 참조.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr"/>
-      <c r="B14" s="31" t="inlineStr"/>
+      <c r="A14" s="29" t="inlineStr"/>
+      <c r="B14" s="30" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>[이미지 파일명 규칙]</t>
         </is>
       </c>
-      <c r="B15" s="29" t="inlineStr"/>
+      <c r="B15" s="28" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>형식</t>
         </is>
       </c>
-      <c r="B16" s="31" t="inlineStr">
+      <c r="B16" s="30" t="inlineStr">
         <is>
           <t>{문항코드}_{슬롯}{순번}.png  (업로드 시 자동 부여)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>슬롯</t>
         </is>
       </c>
-      <c r="B17" s="31" t="inlineStr">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>발문=stem · 보기=opt1~opt4 · 해설=exp · 오답분석=wrong · 학습포인트=lp</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="30" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>예시</t>
         </is>
       </c>
-      <c r="B18" s="31" t="inlineStr">
+      <c r="B18" s="30" t="inlineStr">
         <is>
           <t>elec_A_2022_01_39_lp1.png  (39번 학습포인트 1번 그림)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>참조</t>
         </is>
       </c>
-      <c r="B19" s="31" t="inlineStr">
+      <c r="B19" s="30" t="inlineStr">
         <is>
           <t>셀에는 &lt;img src="elec_A_2022_01_39_lp1.png"&gt; 형태로 본문 어디에나</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="30" t="inlineStr"/>
-      <c r="B20" s="31" t="inlineStr"/>
+      <c r="A20" s="29" t="inlineStr"/>
+      <c r="B20" s="30" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t>[허용 HTML 태그]</t>
         </is>
       </c>
-      <c r="B21" s="29" t="inlineStr"/>
+      <c r="B21" s="28" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="30" t="inlineStr">
+      <c r="A22" s="29" t="inlineStr">
         <is>
           <t>강조/첨자</t>
         </is>
       </c>
-      <c r="B22" s="31" t="inlineStr">
+      <c r="B22" s="30" t="inlineStr">
         <is>
           <t>&lt;strong&gt; &lt;em&gt; &lt;u&gt; &lt;sub&gt; &lt;sup&gt;</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="30" t="inlineStr">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>줄바꿈</t>
         </is>
       </c>
-      <c r="B23" s="31" t="inlineStr">
+      <c r="B23" s="30" t="inlineStr">
         <is>
           <t>&lt;br&gt;</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="30" t="inlineStr">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>그림</t>
         </is>
       </c>
-      <c r="B24" s="31" t="inlineStr">
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t>&lt;img src="파일명"&gt;</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="inlineStr">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t>박스(틀)</t>
         </is>
       </c>
-      <c r="B25" s="31" t="inlineStr">
+      <c r="B25" s="30" t="inlineStr">
         <is>
           <t>&lt;div style="..."&gt; — 아래 표준 스니펫만</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="30" t="inlineStr">
+      <c r="A26" s="29" t="inlineStr">
         <is>
           <t>특수문자</t>
         </is>
       </c>
-      <c r="B26" s="31" t="inlineStr">
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>&amp;lt;는 &lt; · &amp;gt;는 &gt; · &amp;amp;는 &amp;</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="30" t="inlineStr"/>
-      <c r="B27" s="31" t="inlineStr"/>
+      <c r="A27" s="29" t="inlineStr"/>
+      <c r="B27" s="30" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="inlineStr">
+      <c r="A28" s="27" t="inlineStr">
         <is>
           <t>[금지 — 대체 방법]</t>
         </is>
       </c>
-      <c r="B28" s="29" t="inlineStr"/>
+      <c r="B28" s="28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="30" t="inlineStr">
+      <c r="A29" s="29" t="inlineStr">
         <is>
           <t>&lt;ol&gt;&lt;ul&gt;&lt;li&gt;</t>
         </is>
       </c>
-      <c r="B29" s="31" t="inlineStr">
+      <c r="B29" s="30" t="inlineStr">
         <is>
           <t>줄마다 &lt;br&gt;, 번호는 원문자 ①②③④ 로 직접 입력</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="30" t="inlineStr">
+      <c r="A30" s="29" t="inlineStr">
         <is>
           <t>&lt;table&gt;</t>
         </is>
       </c>
-      <c r="B30" s="31" t="inlineStr">
+      <c r="B30" s="30" t="inlineStr">
         <is>
           <t>표·행렬은 LaTeX  $$\begin{array}{...}\end{array}$$</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="inlineStr">
+      <c r="A31" s="29" t="inlineStr">
         <is>
           <t>&lt;p&gt;</t>
         </is>
       </c>
-      <c r="B31" s="31" t="inlineStr">
+      <c r="B31" s="30" t="inlineStr">
         <is>
           <t>문단 구분은 &lt;br&gt;&lt;br&gt;</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="30" t="inlineStr">
+      <c r="A32" s="29" t="inlineStr">
         <is>
           <t>class="..."</t>
         </is>
       </c>
-      <c r="B32" s="31" t="inlineStr">
+      <c r="B32" s="30" t="inlineStr">
         <is>
           <t>모양은 class 금지 → inline style(아래)만</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="30" t="inlineStr"/>
-      <c r="B33" s="31" t="inlineStr"/>
+      <c r="A33" s="29" t="inlineStr"/>
+      <c r="B33" s="30" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="inlineStr">
+      <c r="A34" s="27" t="inlineStr">
         <is>
           <t>[수식 — LaTeX / KaTeX]</t>
         </is>
       </c>
-      <c r="B34" s="29" t="inlineStr"/>
+      <c r="B34" s="28" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="30" t="inlineStr">
+      <c r="A35" s="29" t="inlineStr">
         <is>
           <t>인라인</t>
         </is>
       </c>
-      <c r="B35" s="31" t="inlineStr">
+      <c r="B35" s="30" t="inlineStr">
         <is>
           <t>$ ... $   예) 저항 $R=\dfrac{V}{I}$</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="30" t="inlineStr">
+      <c r="A36" s="29" t="inlineStr">
         <is>
           <t>디스플레이</t>
         </is>
       </c>
-      <c r="B36" s="31" t="inlineStr">
+      <c r="B36" s="30" t="inlineStr">
         <is>
           <t>$$ ... $$   예) $$P=VI=I^2 R$$</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="30" t="inlineStr">
+      <c r="A37" s="29" t="inlineStr">
         <is>
           <t>가능 환경</t>
         </is>
       </c>
-      <c r="B37" s="31" t="inlineStr">
+      <c r="B37" s="30" t="inlineStr">
         <is>
           <t>array · matrix · cases · aligned</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="30" t="inlineStr">
+      <c r="A38" s="29" t="inlineStr">
         <is>
           <t>불가 환경</t>
         </is>
       </c>
-      <c r="B38" s="31" t="inlineStr">
+      <c r="B38" s="30" t="inlineStr">
         <is>
           <t>enumerate · itemize · tabular  (목록은 &lt;br&gt;+원문자)</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="30" t="inlineStr"/>
-      <c r="B39" s="31" t="inlineStr"/>
+      <c r="A39" s="29" t="inlineStr"/>
+      <c r="B39" s="30" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="28" t="inlineStr">
+      <c r="A40" s="27" t="inlineStr">
         <is>
           <t>[박스 표준 스니펫 — inline style]</t>
         </is>
       </c>
-      <c r="B40" s="29" t="inlineStr"/>
+      <c r="B40" s="28" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="30" t="inlineStr">
+      <c r="A41" s="29" t="inlineStr">
         <is>
           <t>핵심공식(초록)</t>
         </is>
       </c>
-      <c r="B41" s="31" t="inlineStr">
+      <c r="B41" s="30" t="inlineStr">
         <is>
           <t>&lt;div style="border:1px solid #34d399;background:#f0fdf4;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt; $$...$$  ... &lt;/div&gt;</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="30" t="inlineStr">
+      <c r="A42" s="29" t="inlineStr">
         <is>
           <t>주의(호박)</t>
         </is>
       </c>
-      <c r="B42" s="31" t="inlineStr">
+      <c r="B42" s="30" t="inlineStr">
         <is>
           <t>&lt;div style="border:1px solid #fbbf24;background:#fffbeb;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt; &lt;strong style="color:#b45309;"&gt;주의&lt;/strong&gt;&lt;br&gt; ... &lt;/div&gt;</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="30" t="inlineStr">
+      <c r="A43" s="29" t="inlineStr">
         <is>
           <t>규칙</t>
         </is>
       </c>
-      <c r="B43" s="31" t="inlineStr">
+      <c r="B43" s="30" t="inlineStr">
         <is>
           <t>style 값 변경·박스 중첩 금지. 독끝 바깥 박스는 앱이 자동(셀에 안 씀).</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="30" t="inlineStr"/>
-      <c r="B44" s="31" t="inlineStr"/>
+      <c r="A44" s="29" t="inlineStr"/>
+      <c r="B44" s="30" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="28" t="inlineStr">
+      <c r="A45" s="27" t="inlineStr">
         <is>
           <t>[제출 전 체크]</t>
         </is>
       </c>
-      <c r="B45" s="29" t="inlineStr"/>
+      <c r="B45" s="28" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="30" t="inlineStr">
+      <c r="A46" s="29" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B46" s="31" t="inlineStr">
+      <c r="B46" s="30" t="inlineStr">
         <is>
           <t>&lt;ol&gt; &lt;ul&gt; &lt;li&gt; &lt;table&gt; &lt;p&gt; 안 썼나?</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="30" t="inlineStr">
+      <c r="A47" s="29" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B47" s="31" t="inlineStr">
+      <c r="B47" s="30" t="inlineStr">
         <is>
           <t>class= 안 썼나? 모양은 전부 style= 인가?</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="30" t="inlineStr">
+      <c r="A48" s="29" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B48" s="31" t="inlineStr">
+      <c r="B48" s="30" t="inlineStr">
         <is>
           <t>번호는 원문자 ①②③ 인가?</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="30" t="inlineStr">
+      <c r="A49" s="29" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B49" s="31" t="inlineStr">
+      <c r="B49" s="30" t="inlineStr">
         <is>
           <t>표는 &lt;table&gt; 아니라 $$\begin{array}$$ 인가?</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="30" t="inlineStr">
+      <c r="A50" s="29" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B50" s="31" t="inlineStr">
+      <c r="B50" s="30" t="inlineStr">
         <is>
           <t>수식은 $…$ / $$…$$ 안에 있나?</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="30" t="inlineStr">
+      <c r="A51" s="29" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B51" s="31" t="inlineStr">
+      <c r="B51" s="30" t="inlineStr">
         <is>
           <t>이미지 파일명이 {문항코드}_{슬롯}{순번}.png 인가?</t>
         </is>

</xml_diff>

<commit_message>
Gray "독끝 학습 Point" box + 색인 sheet + auto-gen sample HTML
- 박스 표준: 핵심공식/주의 2종 폐기 → 회색 「독끝 학습 Point」 단일
- xlsx: 「색인」 시트 추가(번호·문항코드·과목·발문요약, 자동필터) — 문항 빠른 찾기
- build_sample_2022_1_v1.py: 샘플 HTML도 같은 SAMPLES에서 생성(xlsx와 항상 일치)
- 작성규칙서_미리보기.html: ②-2 과목ID(theory/machinery/facility) 추가,
  이미지 파일명 예시 추가·작성자 명명 방식으로 문구 변경, ⑦ 박스 회색 단일화

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/샘플_2022_1회_v1.xlsx
+++ b/data/templates/샘플_2022_1회_v1.xlsx
@@ -9,8 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="문항등록" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성규칙" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="색인" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'색인'!$A$1:$D$11</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -1039,7 +1042,8 @@
       <c r="AG3" s="25" t="inlineStr">
         <is>
           <t>정전용량 공식
-&lt;div style="border:1px solid #34d399;background:#f0fdf4;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;div style="border:1px solid #cbd5e1;background:#f1f5f9;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;strong style="color:#475569;"&gt;독끝 학습 Point&lt;/strong&gt;&lt;br&gt;
 $$C=\dfrac{\varepsilon S}{d}\;[\text{F}]$$
 $\varepsilon$: 유전율[F/m] · $S$: 극판 단면적[m²] · $d$: 극판 간격[m]
 &lt;/div&gt;</t>
@@ -1154,7 +1158,8 @@
       <c r="AE4" s="25" t="inlineStr">
         <is>
           <t>정전에너지 공식
-&lt;div style="border:1px solid #34d399;background:#f0fdf4;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;div style="border:1px solid #cbd5e1;background:#f1f5f9;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;strong style="color:#475569;"&gt;독끝 학습 Point&lt;/strong&gt;&lt;br&gt;
 $$W=\dfrac{1}{2}CV^2\;[\text{J}]$$
 $W$: 정전에너지[J] · $C$: 정전용량[F] · $V$: 전압[V]
 &lt;/div&gt;</t>
@@ -1271,7 +1276,8 @@
       <c r="AE5" s="25" t="inlineStr">
         <is>
           <t>Y 결선에서는 선간전압이 상전압의 $\sqrt{3}$ 배이다.
-&lt;div style="border:1px solid #34d399;background:#f0fdf4;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;div style="border:1px solid #cbd5e1;background:#f1f5f9;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;strong style="color:#475569;"&gt;독끝 학습 Point&lt;/strong&gt;&lt;br&gt;
 $$V_l=\sqrt{3}\,V_p$$
 $V_l$: 선간전압[V] · $V_p$: 상전압[V]
 &lt;/div&gt;</t>
@@ -1395,7 +1401,8 @@
       <c r="AG6" s="25" t="inlineStr">
         <is>
           <t>전력량과 전력
-&lt;div style="border:1px solid #34d399;background:#f0fdf4;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;div style="border:1px solid #cbd5e1;background:#f1f5f9;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;strong style="color:#475569;"&gt;독끝 학습 Point&lt;/strong&gt;&lt;br&gt;
 $$P=\dfrac{W}{t}\;[\text{W}]$$
 $W$: 전력량[J] · $t$: 시간[s] · $P$: 전력[W]
 &lt;/div&gt;</t>
@@ -1518,7 +1525,8 @@
       <c r="AG7" s="25" t="inlineStr">
         <is>
           <t>교류 순시값 표현식
-&lt;div style="border:1px solid #34d399;background:#f0fdf4;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;div style="border:1px solid #cbd5e1;background:#f1f5f9;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;strong style="color:#475569;"&gt;독끝 학습 Point&lt;/strong&gt;&lt;br&gt;
 $$e=V_m\sin(\omega t+\theta)=V_m\sin(2\pi f t+\theta)\;[\text{V}]$$
 $V_m$: 전압 최댓값[V] · $\omega$: 각속도[rad/s] · $\theta$: 위상 · $f$: 주파수[Hz]
 &lt;/div&gt;</t>
@@ -1640,7 +1648,8 @@
       <c r="AG8" s="25" t="inlineStr">
         <is>
           <t>쿨롱의 법칙 (자기장)
-&lt;div style="border:1px solid #34d399;background:#f0fdf4;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;div style="border:1px solid #cbd5e1;background:#f1f5f9;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;strong style="color:#475569;"&gt;독끝 학습 Point&lt;/strong&gt;&lt;br&gt;
 $$F=k\dfrac{m_1 m_2}{r^2}=6.33\times10^{4}\times\dfrac{m_1 m_2}{r^2}\;[\text{N}]$$
 $k$: 쿨롱 상수 $(6.33\times10^4)$ · $m_1,m_2$: 자극의 세기[Wb] · $r$: 거리[m]
 &lt;/div&gt;</t>
@@ -1768,8 +1777,8 @@
       <c r="AG9" s="25" t="inlineStr">
         <is>
           <t>동기 발전기와 전동기는 $L,\,C$ 부하에 대해 반작용 특성이 서로 반대로 발생한다.
-&lt;div style="border:1px solid #fbbf24;background:#fffbeb;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
-&lt;strong style="color:#b45309;"&gt;주의&lt;/strong&gt;&lt;br&gt;
+&lt;div style="border:1px solid #cbd5e1;background:#f1f5f9;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;strong style="color:#475569;"&gt;독끝 학습 Point&lt;/strong&gt;&lt;br&gt;
 발전기의 지상(L)=감자, 전동기의 지상(L)=증자. 발전기 기준으로만 외우면 전동기에서 반대로 틀린다.
 &lt;/div&gt;</t>
         </is>
@@ -1890,7 +1899,8 @@
       <c r="AG10" s="25" t="inlineStr">
         <is>
           <t>변압기의 효율
-&lt;div style="border:1px solid #34d399;background:#f0fdf4;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;div style="border:1px solid #cbd5e1;background:#f1f5f9;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;strong style="color:#475569;"&gt;독끝 학습 Point&lt;/strong&gt;&lt;br&gt;
 $$\eta=\dfrac{P}{P+P_c+P_i}\times100\;[\%]$$
 $P$: 출력 · $P_c$: 동손 · $P_i$: 철손
 &lt;/div&gt;</t>
@@ -2363,7 +2373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2756,7 +2766,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>[박스 표준 스니펫 — inline style]</t>
+          <t>[박스 표준 스니펫 — 독끝 학습 Point · 회색]</t>
         </is>
       </c>
       <c r="B40" s="28" t="inlineStr"/>
@@ -2764,118 +2774,107 @@
     <row r="41">
       <c r="A41" s="29" t="inlineStr">
         <is>
-          <t>핵심공식(초록)</t>
+          <t>스니펫</t>
         </is>
       </c>
       <c r="B41" s="30" t="inlineStr">
         <is>
-          <t>&lt;div style="border:1px solid #34d399;background:#f0fdf4;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt; $$...$$  ... &lt;/div&gt;</t>
+          <t>&lt;div style="border:1px solid #cbd5e1;background:#f1f5f9;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt;
+&lt;strong style="color:#475569;"&gt;독끝 학습 Point&lt;/strong&gt;&lt;br&gt; $$...$$ 또는 텍스트 &lt;/div&gt;</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="29" t="inlineStr">
         <is>
-          <t>주의(호박)</t>
+          <t>규칙</t>
         </is>
       </c>
       <c r="B42" s="30" t="inlineStr">
         <is>
-          <t>&lt;div style="border:1px solid #fbbf24;background:#fffbeb;border-radius:8px;padding:10px 14px;margin:8px 0;"&gt; &lt;strong style="color:#b45309;"&gt;주의&lt;/strong&gt;&lt;br&gt; ... &lt;/div&gt;</t>
+          <t>핵심공식/주의 2종 폐기 → 회색 「독끝 학습 Point」 박스 하나로 통일. style 값 변경·박스 중첩 금지.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="29" t="inlineStr">
-        <is>
-          <t>규칙</t>
-        </is>
-      </c>
-      <c r="B43" s="30" t="inlineStr">
-        <is>
-          <t>style 값 변경·박스 중첩 금지. 독끝 바깥 박스는 앱이 자동(셀에 안 씀).</t>
-        </is>
-      </c>
+      <c r="A43" s="29" t="inlineStr"/>
+      <c r="B43" s="30" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="29" t="inlineStr"/>
-      <c r="B44" s="30" t="inlineStr"/>
+      <c r="A44" s="27" t="inlineStr">
+        <is>
+          <t>[제출 전 체크]</t>
+        </is>
+      </c>
+      <c r="B44" s="28" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="27" t="inlineStr">
-        <is>
-          <t>[제출 전 체크]</t>
-        </is>
-      </c>
-      <c r="B45" s="28" t="inlineStr"/>
+      <c r="A45" s="29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>&lt;ol&gt; &lt;ul&gt; &lt;li&gt; &lt;table&gt; &lt;p&gt; 안 썼나?</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B46" s="30" t="inlineStr">
         <is>
-          <t>&lt;ol&gt; &lt;ul&gt; &lt;li&gt; &lt;table&gt; &lt;p&gt; 안 썼나?</t>
+          <t>class= 안 썼나? 모양은 전부 style= 인가?</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="29" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B47" s="30" t="inlineStr">
         <is>
-          <t>class= 안 썼나? 모양은 전부 style= 인가?</t>
+          <t>번호는 원문자 ①②③ 인가?</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B48" s="30" t="inlineStr">
         <is>
-          <t>번호는 원문자 ①②③ 인가?</t>
+          <t>표는 &lt;table&gt; 아니라 $$\begin{array}$$ 인가?</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B49" s="30" t="inlineStr">
         <is>
-          <t>표는 &lt;table&gt; 아니라 $$\begin{array}$$ 인가?</t>
+          <t>수식은 $…$ / $$…$$ 안에 있나?</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B50" s="30" t="inlineStr">
-        <is>
-          <t>수식은 $…$ / $$…$$ 안에 있나?</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B51" s="30" t="inlineStr">
         <is>
           <t>이미지 파일명이 {문항코드}_{슬롯}{순번}.png 인가?</t>
         </is>
@@ -2884,4 +2883,247 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>번호</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>문항코드</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>과목</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>발문 요약</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="24" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_01</t>
+        </is>
+      </c>
+      <c r="C2" s="24" t="inlineStr">
+        <is>
+          <t>전기이론</t>
+        </is>
+      </c>
+      <c r="D2" s="25" t="inlineStr">
+        <is>
+          <t>콘덴서의 정전용량에 대한 설명으로 틀린 것은?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_02</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>전기이론</t>
+        </is>
+      </c>
+      <c r="D3" s="25" t="inlineStr">
+        <is>
+          <t>정전에너지 W[\text{J}] 를 구하는 식으로 옳은 것은? (단, C 는 콘덴…</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_05</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>전기이론</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>평형 3상 교류회로에서 Y결선할 때 선간전압 V_l 과 상전압 V_p 의 관계는?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_07</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>전기이론</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>20분간 876{,}000[\text{J}] 의 일을 할 때 전력은 약 몇 [\t…</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_11</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>전기이론</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>다음 전압 파형의 주파수는 약 몇 [\text{Hz}] 인가? e=100\sin\…</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_13</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>전기이론</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>m_1=4\times10^{-5}[\text{Wb}], m_2=6\times10^…</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_23</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>전기기기</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>동기 전동기 전기자 반작용에 대한 설명이다. 공급전압에 대한 앞선 전류의 전기자 …</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_32</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>전기기기</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>200[\text{kVA}] 의 단상 변압기가 있다. 철손이 1.6[\text{k…</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_39</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>전기설비</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>역병렬 결합의 SCR의 특성과 같은 반도체 소자는?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>elec_A_2022_01_60</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>전기설비</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>소맥분, 전분 기타 가연성의 분진이 존재하는 곳의 저압 옥내 배선 공사 방법에 해…</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>